<commit_message>
feat: Add bulk confirmation for exact reconciliation deposits
- Implemented a new feature to confirm all exact reconciliation deposits in the Capital Call policy.
- Added a button in the reconciliation panel to trigger the confirmation modal for matched deposits.
- Created a modal to summarize the actions that will be taken when confirming all matched deposits.
- Updated the RemittanceReconciliationAgent to handle ambiguous accounts and provide clearer reasoning for reviewers.
- Enhanced the reconciliation report generation to include coverage options for full and sample outputs.
- Updated routes to include the new confirmation action for exact deposits.
- Added Cucumber tests to validate the new bulk confirmation functionality.
- Improved tooltips and labels for clarity in the reconciliation UI.
</commit_message>
<xml_diff>
--- a/public/sample_uploads/remittance_recon_call_719_axis.xlsx
+++ b/public/sample_uploads/remittance_recon_call_719_axis.xlsx
@@ -327,12 +327,12 @@
   <sheetPr>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
   <cols>
     <col width="66.0" min="1" max="1" bestFit="1" customWidth="1"/>
     <col width="20.900000000000002" min="2" max="2" bestFit="1" customWidth="1"/>
-    <col width="40.7" min="3" max="3" bestFit="1" customWidth="1"/>
+    <col width="45.1" min="3" max="3" bestFit="1" customWidth="1"/>
     <col width="16.5" min="4" max="4" bestFit="1" customWidth="1"/>
     <col width="16.5" min="5" max="5" bestFit="1" customWidth="1"/>
   </cols>
@@ -528,7 +528,7 @@
       </c>
       <c r="C11" s="0" t="inlineStr">
         <is>
-          <t>TRF/NOBODY MATCHES ME/TRANSFER</t>
+          <t>MOB/TPFT/G/50100133674524</t>
         </is>
       </c>
       <c r="D11" s="0" t="n">
@@ -551,11 +551,11 @@
       </c>
       <c r="C12" s="0" t="inlineStr">
         <is>
-          <t>926040079793295 : Closure Proceeds</t>
+          <t>MOB/TPFT/H/00601100066619</t>
         </is>
       </c>
       <c r="D12" s="0" t="n">
-        <v>3003452.1</v>
+        <v>100000.0</v>
       </c>
       <c r="E12" s="0" t="inlineStr">
         <is>
@@ -574,13 +574,1669 @@
       </c>
       <c r="C13" s="0" t="inlineStr">
         <is>
+          <t>MOB/TPFT/I/50200007064902</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="n">
+        <v>100000.0</v>
+      </c>
+      <c r="E13" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/J/50100035238824</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="n">
+        <v>100000.0</v>
+      </c>
+      <c r="E14" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/L/00142790000324</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="n">
+        <v>200000.0</v>
+      </c>
+      <c r="E15" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/M/50132010049181</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="n">
+        <v>100000.0</v>
+      </c>
+      <c r="E16" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/N/10324773718</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="n">
+        <v>500000.0</v>
+      </c>
+      <c r="E17" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>TRF/O/TRANSFER</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="n">
+        <v>5000000.0</v>
+      </c>
+      <c r="E18" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/P/00602480038037</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="n">
+        <v>300000.0</v>
+      </c>
+      <c r="E19" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/Q/50100225695725</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="n">
+        <v>125000.0</v>
+      </c>
+      <c r="E20" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/R/50100263909150</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="n">
+        <v>200000.0</v>
+      </c>
+      <c r="E21" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/S/00601100058003</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="n">
+        <v>200000.0</v>
+      </c>
+      <c r="E22" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/T/50100190500177</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="n">
+        <v>200000.0</v>
+      </c>
+      <c r="E23" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/U/50100279243414</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="n">
+        <v>200000.0</v>
+      </c>
+      <c r="E24" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/V/50200039466179</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="n">
+        <v>200000.0</v>
+      </c>
+      <c r="E25" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="B26" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/W/50100140518099</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="n">
+        <v>200000.0</v>
+      </c>
+      <c r="E26" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="B27" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/X/02911610049610</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="n">
+        <v>300000.0</v>
+      </c>
+      <c r="E27" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="B28" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/Y/50200033085962</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="n">
+        <v>3000000.0</v>
+      </c>
+      <c r="E28" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="B29" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/Z/00600340080091</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="n">
+        <v>2000000.0</v>
+      </c>
+      <c r="E29" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="B30" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/AA/50100169434100</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="n">
+        <v>200000.0</v>
+      </c>
+      <c r="E30" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="B31" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/AB/50100265170502</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="n">
+        <v>200000.0</v>
+      </c>
+      <c r="E31" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="B32" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/AC/50100104765675</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="n">
+        <v>1500000.0</v>
+      </c>
+      <c r="E32" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="B33" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/AD/00591050008474</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="n">
+        <v>100000.0</v>
+      </c>
+      <c r="E33" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="B34" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/AE/50200062960056</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="n">
+        <v>100000.0</v>
+      </c>
+      <c r="E34" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="B35" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/AF/50100452472153</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="n">
+        <v>100000.0</v>
+      </c>
+      <c r="E35" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="B36" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/AG/15772030011954</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="n">
+        <v>200000.0</v>
+      </c>
+      <c r="E36" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="B37" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/AH/05227630000193</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="n">
+        <v>200000.0</v>
+      </c>
+      <c r="E37" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="B38" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/AI/50200042386031</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="n">
+        <v>100000.0</v>
+      </c>
+      <c r="E38" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="B39" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/AJ/50100129316544</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="n">
+        <v>200000.0</v>
+      </c>
+      <c r="E39" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="B40" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/AK/50100174601251</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="n">
+        <v>750000.0</v>
+      </c>
+      <c r="E40" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="B41" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/AL/50200024385240</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="n">
+        <v>200000.0</v>
+      </c>
+      <c r="E41" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="B42" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/AM/50200026492711</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="n">
+        <v>100000.0</v>
+      </c>
+      <c r="E42" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="B43" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/AN/15772030008891</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="n">
+        <v>150000.0</v>
+      </c>
+      <c r="E43" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="B44" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/AO/15772030008909</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="n">
+        <v>150000.0</v>
+      </c>
+      <c r="E44" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="B45" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/AP/61159199180</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="n">
+        <v>200000.0</v>
+      </c>
+      <c r="E45" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="B46" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/AQ/50100334040562</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="n">
+        <v>500000.0</v>
+      </c>
+      <c r="E46" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="B47" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/AR/50200019917741</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="n">
+        <v>200000.0</v>
+      </c>
+      <c r="E47" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="B48" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/AS/02401300000354</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="n">
+        <v>200000.0</v>
+      </c>
+      <c r="E48" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="B49" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/AT/000405071553</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="n">
+        <v>500000.0</v>
+      </c>
+      <c r="E49" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="B50" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/AU/50100226072314</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="n">
+        <v>200000.0</v>
+      </c>
+      <c r="E50" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="B51" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/AV/50100212286171</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="n">
+        <v>100000.0</v>
+      </c>
+      <c r="E51" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="B52" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C52" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/AW/50100213461809</t>
+        </is>
+      </c>
+      <c r="D52" s="0" t="n">
+        <v>100000.0</v>
+      </c>
+      <c r="E52" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="B53" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C53" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/AX/918010022821819</t>
+        </is>
+      </c>
+      <c r="D53" s="0" t="n">
+        <v>100000.0</v>
+      </c>
+      <c r="E53" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="B54" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C54" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/AY/50100225371522</t>
+        </is>
+      </c>
+      <c r="D54" s="0" t="n">
+        <v>200000.0</v>
+      </c>
+      <c r="E54" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="0" t="n">
+        <v>51</v>
+      </c>
+      <c r="B55" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C55" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/AZ/4912642396</t>
+        </is>
+      </c>
+      <c r="D55" s="0" t="n">
+        <v>200000.0</v>
+      </c>
+      <c r="E55" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="0" t="n">
+        <v>52</v>
+      </c>
+      <c r="B56" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C56" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/BA/50200024323031</t>
+        </is>
+      </c>
+      <c r="D56" s="0" t="n">
+        <v>200000.0</v>
+      </c>
+      <c r="E56" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="0" t="n">
+        <v>53</v>
+      </c>
+      <c r="B57" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C57" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/BB/50200034109309</t>
+        </is>
+      </c>
+      <c r="D57" s="0" t="n">
+        <v>100000.0</v>
+      </c>
+      <c r="E57" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="0" t="n">
+        <v>54</v>
+      </c>
+      <c r="B58" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C58" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/BC/10503338670</t>
+        </is>
+      </c>
+      <c r="D58" s="0" t="n">
+        <v>500000.0</v>
+      </c>
+      <c r="E58" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="0" t="n">
+        <v>55</v>
+      </c>
+      <c r="B59" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C59" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/BD/50100196328630</t>
+        </is>
+      </c>
+      <c r="D59" s="0" t="n">
+        <v>200000.0</v>
+      </c>
+      <c r="E59" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="0" t="n">
+        <v>56</v>
+      </c>
+      <c r="B60" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C60" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/BE/10050170172</t>
+        </is>
+      </c>
+      <c r="D60" s="0" t="n">
+        <v>100000.0</v>
+      </c>
+      <c r="E60" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="0" t="n">
+        <v>57</v>
+      </c>
+      <c r="B61" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C61" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/BF/10050170310</t>
+        </is>
+      </c>
+      <c r="D61" s="0" t="n">
+        <v>100000.0</v>
+      </c>
+      <c r="E61" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="0" t="n">
+        <v>58</v>
+      </c>
+      <c r="B62" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C62" s="0" t="inlineStr">
+        <is>
+          <t>TRF/BG/TRANSFER</t>
+        </is>
+      </c>
+      <c r="D62" s="0" t="n">
+        <v>200000.0</v>
+      </c>
+      <c r="E62" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="0" t="n">
+        <v>59</v>
+      </c>
+      <c r="B63" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C63" s="0" t="inlineStr">
+        <is>
+          <t>TRF/BH/TRANSFER</t>
+        </is>
+      </c>
+      <c r="D63" s="0" t="n">
+        <v>100000.0</v>
+      </c>
+      <c r="E63" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="0" t="n">
+        <v>60</v>
+      </c>
+      <c r="B64" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C64" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/BI/50200031714742</t>
+        </is>
+      </c>
+      <c r="D64" s="0" t="n">
+        <v>100000.0</v>
+      </c>
+      <c r="E64" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="0" t="n">
+        <v>61</v>
+      </c>
+      <c r="B65" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C65" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/BJ/50200032982656</t>
+        </is>
+      </c>
+      <c r="D65" s="0" t="n">
+        <v>195470.0</v>
+      </c>
+      <c r="E65" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="0" t="n">
+        <v>62</v>
+      </c>
+      <c r="B66" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C66" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/BK/50200032841632</t>
+        </is>
+      </c>
+      <c r="D66" s="0" t="n">
+        <v>191680.0</v>
+      </c>
+      <c r="E66" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="0" t="n">
+        <v>63</v>
+      </c>
+      <c r="B67" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C67" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/BL/50100269866900</t>
+        </is>
+      </c>
+      <c r="D67" s="0" t="n">
+        <v>100000.0</v>
+      </c>
+      <c r="E67" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="0" t="n">
+        <v>64</v>
+      </c>
+      <c r="B68" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C68" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/BM/1787411939</t>
+        </is>
+      </c>
+      <c r="D68" s="0" t="n">
+        <v>240400.0</v>
+      </c>
+      <c r="E68" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="0" t="n">
+        <v>65</v>
+      </c>
+      <c r="B69" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C69" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/BN/001501005380</t>
+        </is>
+      </c>
+      <c r="D69" s="0" t="n">
+        <v>100000.0</v>
+      </c>
+      <c r="E69" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="0" t="n">
+        <v>66</v>
+      </c>
+      <c r="B70" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C70" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/BO/50100201521237</t>
+        </is>
+      </c>
+      <c r="D70" s="0" t="n">
+        <v>100000.0</v>
+      </c>
+      <c r="E70" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="0" t="n">
+        <v>67</v>
+      </c>
+      <c r="B71" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C71" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/BP/50100090651508</t>
+        </is>
+      </c>
+      <c r="D71" s="0" t="n">
+        <v>7000268.51</v>
+      </c>
+      <c r="E71" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="0" t="n">
+        <v>68</v>
+      </c>
+      <c r="B72" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C72" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/BQ/50100293012215</t>
+        </is>
+      </c>
+      <c r="D72" s="0" t="n">
+        <v>2360290.0</v>
+      </c>
+      <c r="E72" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="0" t="n">
+        <v>69</v>
+      </c>
+      <c r="B73" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C73" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/BR/004103000025133</t>
+        </is>
+      </c>
+      <c r="D73" s="0" t="n">
+        <v>1888230.0</v>
+      </c>
+      <c r="E73" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="0" t="n">
+        <v>70</v>
+      </c>
+      <c r="B74" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C74" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/BS/602320013480</t>
+        </is>
+      </c>
+      <c r="D74" s="0" t="n">
+        <v>100000.0</v>
+      </c>
+      <c r="E74" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="0" t="n">
+        <v>71</v>
+      </c>
+      <c r="B75" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C75" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/ARUN GUPTA HOLDING/3338880980</t>
+        </is>
+      </c>
+      <c r="D75" s="0" t="n">
+        <v>863500.0</v>
+      </c>
+      <c r="E75" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="0" t="n">
+        <v>72</v>
+      </c>
+      <c r="B76" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C76" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/A/50100033849984</t>
+        </is>
+      </c>
+      <c r="D76" s="0" t="n">
+        <v>100000.0</v>
+      </c>
+      <c r="E76" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="0" t="n">
+        <v>73</v>
+      </c>
+      <c r="B77" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C77" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/ARUN GUPTA HOLDING/3388000182</t>
+        </is>
+      </c>
+      <c r="D77" s="0" t="n">
+        <v>600000.0</v>
+      </c>
+      <c r="E77" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="0" t="n">
+        <v>74</v>
+      </c>
+      <c r="B78" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C78" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/INVESTOR 11/2346898808</t>
+        </is>
+      </c>
+      <c r="D78" s="0" t="n">
+        <v>10000.0</v>
+      </c>
+      <c r="E78" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="0" t="n">
+        <v>75</v>
+      </c>
+      <c r="B79" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C79" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/ARUN GUPTA HOLDING/3338880980</t>
+        </is>
+      </c>
+      <c r="D79" s="0" t="n">
+        <v>100000.0</v>
+      </c>
+      <c r="E79" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="0" t="n">
+        <v>76</v>
+      </c>
+      <c r="B80" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C80" s="0" t="inlineStr">
+        <is>
+          <t>TRF/AWESOME ACCOUNTING/TRANSFER</t>
+        </is>
+      </c>
+      <c r="D80" s="0" t="n">
+        <v>200000.0</v>
+      </c>
+      <c r="E80" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="0" t="n">
+        <v>77</v>
+      </c>
+      <c r="B81" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C81" s="0" t="inlineStr">
+        <is>
+          <t>MOB/TPFT/ARUN GUPTA HOLDING/3338880980</t>
+        </is>
+      </c>
+      <c r="D81" s="0" t="n">
+        <v>500000.0</v>
+      </c>
+      <c r="E81" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="0" t="n">
+        <v>78</v>
+      </c>
+      <c r="B82" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C82" s="0" t="inlineStr">
+        <is>
+          <t>TRF/AAA/TRANSFER</t>
+        </is>
+      </c>
+      <c r="D82" s="0" t="n">
+        <v>200000.0</v>
+      </c>
+      <c r="E82" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="0" t="n">
+        <v>79</v>
+      </c>
+      <c r="B83" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C83" s="0" t="inlineStr">
+        <is>
+          <t>TRF/NOBODY MATCHES ME/TRANSFER</t>
+        </is>
+      </c>
+      <c r="D83" s="0" t="n">
+        <v>100000.0</v>
+      </c>
+      <c r="E83" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="0" t="n">
+        <v>80</v>
+      </c>
+      <c r="B84" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C84" s="0" t="inlineStr">
+        <is>
+          <t>926040079793295 : Closure Proceeds</t>
+        </is>
+      </c>
+      <c r="D84" s="0" t="n">
+        <v>3003452.1</v>
+      </c>
+      <c r="E84" s="0" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="0" t="n">
+        <v>81</v>
+      </c>
+      <c r="B85" s="0" t="inlineStr">
+        <is>
+          <t>25/02/2025</t>
+        </is>
+      </c>
+      <c r="C85" s="0" t="inlineStr">
+        <is>
           <t>SGB/3101499/FUND 1/Transfer</t>
         </is>
       </c>
-      <c r="D13" s="0" t="n">
+      <c r="D85" s="0" t="n">
         <v>1900000.0</v>
       </c>
-      <c r="E13" s="0" t="inlineStr">
+      <c r="E85" s="0" t="inlineStr">
         <is>
           <t>DR</t>
         </is>

</xml_diff>